<commit_message>
add: Retorno Pago Sri
</commit_message>
<xml_diff>
--- a/api/src/main/resources/importaciones/Base1RepDinardap.xlsx
+++ b/api/src/main/resources/importaciones/Base1RepDinardap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC08EAD-EC40-4233-8375-DCD707F5A286}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7463F89F-CF7F-4CCC-91EC-F06D19CB533D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{CAF234AD-E9C7-413A-814C-96349B608FC2}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$B$1:$B$1141</definedName>
   </definedNames>
-  <calcPr calcId="191029" refMode="R1C1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -15255,15 +15255,9 @@
       <c r="E110" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F110" s="3">
-        <v>23</v>
-      </c>
-      <c r="G110" s="3">
-        <v>2</v>
-      </c>
-      <c r="H110" s="3">
-        <v>50</v>
-      </c>
+      <c r="F110" s="3"/>
+      <c r="G110" s="3"/>
+      <c r="H110" s="3"/>
       <c r="I110" s="4" t="s">
         <v>406</v>
       </c>
@@ -16617,15 +16611,9 @@
       <c r="E149" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F149" s="3">
-        <v>23</v>
-      </c>
-      <c r="G149" s="3">
-        <v>2</v>
-      </c>
-      <c r="H149" s="3">
-        <v>50</v>
-      </c>
+      <c r="F149" s="3"/>
+      <c r="G149" s="3"/>
+      <c r="H149" s="3"/>
       <c r="I149" s="4" t="s">
         <v>406</v>
       </c>
@@ -27587,15 +27575,9 @@
       <c r="E468" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F468" s="3">
-        <v>12</v>
-      </c>
-      <c r="G468" s="3">
-        <v>7</v>
-      </c>
-      <c r="H468" s="3">
-        <v>2</v>
-      </c>
+      <c r="F468" s="3"/>
+      <c r="G468" s="3"/>
+      <c r="H468" s="3"/>
       <c r="I468" s="4" t="s">
         <v>625</v>
       </c>
@@ -31211,15 +31193,9 @@
       <c r="E573" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F573" s="3">
-        <v>12</v>
-      </c>
-      <c r="G573" s="3">
-        <v>7</v>
-      </c>
-      <c r="H573" s="3">
-        <v>2</v>
-      </c>
+      <c r="F573" s="3"/>
+      <c r="G573" s="3"/>
+      <c r="H573" s="3"/>
       <c r="I573" s="4" t="s">
         <v>625</v>
       </c>
@@ -36489,15 +36465,9 @@
       <c r="E725" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F725" s="3">
-        <v>9</v>
-      </c>
-      <c r="G725" s="3">
-        <v>10</v>
-      </c>
-      <c r="H725" s="3">
-        <v>2</v>
-      </c>
+      <c r="F725" s="3"/>
+      <c r="G725" s="3"/>
+      <c r="H725" s="3"/>
       <c r="I725" s="4" t="s">
         <v>2327</v>
       </c>
@@ -41987,15 +41957,9 @@
       <c r="E882" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F882" s="3">
-        <v>12</v>
-      </c>
-      <c r="G882" s="3">
-        <v>7</v>
-      </c>
-      <c r="H882" s="3">
-        <v>2</v>
-      </c>
+      <c r="F882" s="3"/>
+      <c r="G882" s="3"/>
+      <c r="H882" s="3"/>
       <c r="I882" s="4" t="s">
         <v>625</v>
       </c>
@@ -47055,15 +47019,9 @@
       <c r="E1028" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F1028" s="3">
-        <v>11</v>
-      </c>
-      <c r="G1028" s="3">
-        <v>1</v>
-      </c>
-      <c r="H1028" s="3">
-        <v>5</v>
-      </c>
+      <c r="F1028" s="3"/>
+      <c r="G1028" s="3"/>
+      <c r="H1028" s="3"/>
       <c r="I1028" s="4" t="s">
         <v>3244</v>
       </c>
@@ -49611,15 +49569,9 @@
       <c r="E1103" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1103" s="3">
-        <v>12</v>
-      </c>
-      <c r="G1103" s="3">
-        <v>7</v>
-      </c>
-      <c r="H1103" s="3">
-        <v>2</v>
-      </c>
+      <c r="F1103" s="3"/>
+      <c r="G1103" s="3"/>
+      <c r="H1103" s="3"/>
       <c r="I1103" s="4" t="s">
         <v>625</v>
       </c>
@@ -50903,15 +50855,9 @@
       <c r="E1140" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1140" s="3">
-        <v>12</v>
-      </c>
-      <c r="G1140" s="3">
-        <v>7</v>
-      </c>
-      <c r="H1140" s="3">
-        <v>2</v>
-      </c>
+      <c r="F1140" s="3"/>
+      <c r="G1140" s="3"/>
+      <c r="H1140" s="3"/>
       <c r="I1140" s="4" t="s">
         <v>625</v>
       </c>

</xml_diff>